<commit_message>
remove legal metadata from ontology
</commit_message>
<xml_diff>
--- a/data/daschland_ontology/lists/list.xlsx
+++ b/data/daschland_ontology/lists/list.xlsx
@@ -1,29 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11028"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/noemivillars-amberg/Documents/daschland-scripts/daschland_ontology/lists/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/noraammann/Documents/Cloned_GitHub/0854-daschland-scripts/data/daschland_ontology/lists/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{418A1BC1-A9CB-5C48-9418-A65760F13291}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0884FDFD-7B16-F84D-A358-6AF08597841D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9380" yWindow="620" windowWidth="58460" windowHeight="26380" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="License List" sheetId="1" r:id="rId1"/>
-    <sheet name="Event Type List" sheetId="2" r:id="rId2"/>
-    <sheet name="Role List" sheetId="3" r:id="rId3"/>
-    <sheet name="Keyword List" sheetId="4" r:id="rId4"/>
+    <sheet name="Event Type List" sheetId="2" r:id="rId1"/>
+    <sheet name="Role List" sheetId="3" r:id="rId2"/>
+    <sheet name="Keyword List" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="635" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="579" uniqueCount="220">
   <si>
     <t>ID (optional)</t>
   </si>
@@ -40,68 +39,6 @@
     <t>fr_1</t>
   </si>
   <si>
-    <t>License</t>
-  </si>
-  <si>
-    <t>Licence</t>
-  </si>
-  <si>
-    <t>LIC_001</t>
-  </si>
-  <si>
-    <t>CC0 1.0</t>
-  </si>
-  <si>
-    <t>LIC_002</t>
-  </si>
-  <si>
-    <t>CC BY 4.0</t>
-  </si>
-  <si>
-    <t>LIC_003</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color indexed="8"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>CC BY-SA 4.0</t>
-    </r>
-  </si>
-  <si>
-    <t>LIC_004</t>
-  </si>
-  <si>
-    <t>CC BY-NC 4.0</t>
-  </si>
-  <si>
-    <t>LIC_005</t>
-  </si>
-  <si>
-    <t>CC BY-NC-SA 4.0</t>
-  </si>
-  <si>
-    <t>LIC_006</t>
-  </si>
-  <si>
-    <t>CC BY-ND 4.0</t>
-  </si>
-  <si>
-    <t>LIC_007</t>
-  </si>
-  <si>
-    <t>CC BY-NC-ND 4.0</t>
-  </si>
-  <si>
-    <t>LIC_008</t>
-  </si>
-  <si>
-    <t>PDM 1.0</t>
-  </si>
-  <si>
     <t>en_2</t>
   </si>
   <si>
@@ -705,25 +642,10 @@
     <t>Onirique</t>
   </si>
   <si>
-    <t>LIC_009</t>
-  </si>
-  <si>
-    <t>Public Domain</t>
-  </si>
-  <si>
-    <t>Domaine Public</t>
-  </si>
-  <si>
     <t>en_comments</t>
   </si>
   <si>
     <t>fr_comments</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Licenses used in the project </t>
-  </si>
-  <si>
-    <t>Licences en utilisation dans le projet</t>
   </si>
   <si>
     <t>The events of Alice in Wonderland are subdivised into four main types and their subdivisions. This list explores the possibility of hierarchical controlled vocabularies.</t>
@@ -837,7 +759,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -846,7 +768,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1982,230 +1903,6 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" customHeight="1" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="3" width="10.83203125" style="1" customWidth="1"/>
-    <col min="4" max="5" width="15" style="1" customWidth="1"/>
-    <col min="6" max="7" width="32" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="10.83203125" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="10" t="s">
-        <v>227</v>
-      </c>
-      <c r="G1" s="11" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="3"/>
-      <c r="B2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="9" t="s">
-        <v>229</v>
-      </c>
-      <c r="G2" s="12" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="8" t="s">
-        <v>224</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>225</v>
-      </c>
-      <c r="E11" s="8" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="D5" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="E5" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait"/>
-  <headerFooter>
-    <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -2238,31 +1935,31 @@
         <v>4</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="J1" s="10" t="s">
-        <v>227</v>
-      </c>
-      <c r="K1" s="11" t="s">
-        <v>228</v>
+        <v>8</v>
+      </c>
+      <c r="J1" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="K1" s="10" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="5"/>
       <c r="B2" s="4" t="s">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
@@ -2270,28 +1967,28 @@
       <c r="G2" s="5"/>
       <c r="H2" s="5"/>
       <c r="I2" s="5"/>
-      <c r="J2" s="9" t="s">
-        <v>231</v>
-      </c>
-      <c r="K2" s="9" t="s">
-        <v>234</v>
+      <c r="J2" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="K2" s="8" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="5"/>
@@ -2300,144 +1997,144 @@
     </row>
     <row r="4" spans="1:11" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="H4" s="5"/>
       <c r="I4" s="5"/>
     </row>
     <row r="5" spans="1:11" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="H5" s="5"/>
       <c r="I5" s="5"/>
     </row>
     <row r="6" spans="1:11" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="H6" s="5"/>
       <c r="I6" s="5"/>
     </row>
     <row r="7" spans="1:11" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="H7" s="5"/>
       <c r="I7" s="5"/>
     </row>
     <row r="8" spans="1:11" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>43</v>
+        <v>25</v>
       </c>
       <c r="B8" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G8" s="4" t="s">
         <v>27</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>45</v>
       </c>
       <c r="H8" s="5"/>
       <c r="I8" s="5"/>
     </row>
     <row r="9" spans="1:11" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>47</v>
+        <v>29</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>47</v>
+        <v>29</v>
       </c>
       <c r="F9" s="5"/>
       <c r="G9" s="5"/>
@@ -2446,94 +2143,94 @@
     </row>
     <row r="10" spans="1:11" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>47</v>
+        <v>29</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>47</v>
+        <v>29</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="H10" s="5"/>
       <c r="I10" s="5"/>
     </row>
     <row r="11" spans="1:11" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>47</v>
+        <v>29</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>47</v>
+        <v>29</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="H11" s="5"/>
       <c r="I11" s="5"/>
     </row>
     <row r="12" spans="1:11" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
-        <v>53</v>
+        <v>35</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>47</v>
+        <v>29</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>47</v>
+        <v>29</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>54</v>
+        <v>36</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="H12" s="5"/>
       <c r="I12" s="5"/>
     </row>
     <row r="13" spans="1:11" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>57</v>
+        <v>39</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="F13" s="5"/>
       <c r="G13" s="5"/>
@@ -2542,123 +2239,123 @@
     </row>
     <row r="14" spans="1:11" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
-        <v>59</v>
+        <v>41</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>57</v>
+        <v>39</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="F14" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="G14" s="14" t="s">
-        <v>60</v>
+        <v>40</v>
+      </c>
+      <c r="F14" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="G14" s="13" t="s">
+        <v>42</v>
       </c>
       <c r="H14" s="5"/>
       <c r="I14" s="5"/>
     </row>
     <row r="15" spans="1:11" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>57</v>
+        <v>39</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>62</v>
+        <v>44</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>62</v>
+        <v>44</v>
       </c>
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
     </row>
     <row r="16" spans="1:11" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
-        <v>63</v>
+        <v>45</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>57</v>
+        <v>39</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>62</v>
+        <v>44</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>62</v>
+        <v>44</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>64</v>
+        <v>46</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>65</v>
+        <v>47</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>57</v>
+        <v>39</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
       <c r="H17" s="5"/>
       <c r="I17" s="5"/>
     </row>
     <row r="18" spans="1:9" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
-        <v>69</v>
+        <v>51</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>71</v>
+        <v>53</v>
       </c>
       <c r="F18" s="5"/>
       <c r="G18" s="5"/>
@@ -2674,7 +2371,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -2704,62 +2401,62 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="10" t="s">
-        <v>227</v>
-      </c>
-      <c r="G1" s="11" t="s">
-        <v>228</v>
+      <c r="F1" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3"/>
       <c r="B2" s="2" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>73</v>
+        <v>55</v>
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
-      <c r="F2" s="9" t="s">
-        <v>232</v>
-      </c>
-      <c r="G2" s="12" t="s">
-        <v>233</v>
+      <c r="F2" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="G2" s="11" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>74</v>
+        <v>56</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>73</v>
+        <v>55</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>75</v>
+        <v>57</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>77</v>
+        <v>59</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>73</v>
+        <v>55</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>79</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -2813,7 +2510,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:U140"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -2857,28 +2554,28 @@
         <v>4</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>80</v>
+        <v>62</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="L1" s="10" t="s">
-        <v>227</v>
-      </c>
-      <c r="M1" s="11" t="s">
-        <v>228</v>
+        <v>63</v>
+      </c>
+      <c r="L1" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="M1" s="10" t="s">
+        <v>207</v>
       </c>
       <c r="N1" s="5"/>
       <c r="O1" s="5"/>
@@ -2892,10 +2589,10 @@
     <row r="2" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="5"/>
       <c r="B2" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
@@ -2906,10 +2603,10 @@
       <c r="J2" s="5"/>
       <c r="K2" s="5"/>
       <c r="L2" s="1" t="s">
-        <v>236</v>
-      </c>
-      <c r="M2" s="13" t="s">
-        <v>235</v>
+        <v>213</v>
+      </c>
+      <c r="M2" s="12" t="s">
+        <v>212</v>
       </c>
       <c r="N2" s="5"/>
       <c r="O2" s="5"/>
@@ -2922,19 +2619,19 @@
     </row>
     <row r="3" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
-        <v>84</v>
+        <v>66</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="5"/>
@@ -2942,11 +2639,11 @@
       <c r="I3" s="5"/>
       <c r="J3" s="5"/>
       <c r="K3" s="5"/>
-      <c r="L3" s="13" t="s">
-        <v>241</v>
-      </c>
-      <c r="M3" s="13" t="s">
-        <v>242</v>
+      <c r="L3" s="12" t="s">
+        <v>218</v>
+      </c>
+      <c r="M3" s="12" t="s">
+        <v>219</v>
       </c>
       <c r="N3" s="5"/>
       <c r="O3" s="5"/>
@@ -2959,25 +2656,25 @@
     </row>
     <row r="4" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
-        <v>87</v>
+        <v>69</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>89</v>
+        <v>71</v>
       </c>
       <c r="H4" s="5"/>
       <c r="I4" s="5"/>
@@ -2996,31 +2693,31 @@
     </row>
     <row r="5" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>89</v>
+        <v>71</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>92</v>
+        <v>74</v>
       </c>
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
@@ -3037,31 +2734,31 @@
     </row>
     <row r="6" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>93</v>
+        <v>75</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>89</v>
+        <v>71</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
@@ -3078,31 +2775,31 @@
     </row>
     <row r="7" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>89</v>
+        <v>71</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>96</v>
+        <v>78</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>96</v>
+        <v>78</v>
       </c>
       <c r="J7" s="5"/>
       <c r="K7" s="5"/>
@@ -3119,31 +2816,31 @@
     </row>
     <row r="8" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>97</v>
+        <v>79</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>89</v>
+        <v>71</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>99</v>
+        <v>81</v>
       </c>
       <c r="J8" s="5"/>
       <c r="K8" s="5"/>
@@ -3160,25 +2857,25 @@
     </row>
     <row r="9" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="H9" s="5"/>
       <c r="I9" s="5"/>
@@ -3197,31 +2894,31 @@
     </row>
     <row r="10" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D10" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="I10" s="6" t="s">
         <v>85</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="G10" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="H10" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="I10" s="6" t="s">
-        <v>103</v>
       </c>
       <c r="J10" s="5"/>
       <c r="K10" s="5"/>
@@ -3238,31 +2935,31 @@
     </row>
     <row r="11" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
-        <v>104</v>
+        <v>86</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="J11" s="5"/>
       <c r="K11" s="5"/>
@@ -3279,25 +2976,25 @@
     </row>
     <row r="12" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
-        <v>105</v>
+        <v>87</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>106</v>
+        <v>88</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>107</v>
+        <v>89</v>
       </c>
       <c r="H12" s="5"/>
       <c r="I12" s="5"/>
@@ -3316,31 +3013,31 @@
     </row>
     <row r="13" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
-        <v>108</v>
+        <v>90</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>106</v>
+        <v>88</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>107</v>
+        <v>89</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>110</v>
+        <v>92</v>
       </c>
       <c r="J13" s="5"/>
       <c r="K13" s="5"/>
@@ -3357,37 +3054,37 @@
     </row>
     <row r="14" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
-        <v>111</v>
+        <v>93</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>106</v>
+        <v>88</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>107</v>
+        <v>89</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>110</v>
+        <v>92</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>112</v>
+        <v>94</v>
       </c>
       <c r="K14" s="6" t="s">
-        <v>113</v>
+        <v>95</v>
       </c>
       <c r="L14" s="5"/>
       <c r="M14" s="5"/>
@@ -3402,37 +3099,37 @@
     </row>
     <row r="15" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
-        <v>114</v>
+        <v>96</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>106</v>
+        <v>88</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>107</v>
+        <v>89</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>110</v>
+        <v>92</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>116</v>
+        <v>98</v>
       </c>
       <c r="L15" s="5"/>
       <c r="M15" s="5"/>
@@ -3447,31 +3144,31 @@
     </row>
     <row r="16" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
-        <v>117</v>
+        <v>99</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>106</v>
+        <v>88</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>107</v>
+        <v>89</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="I16" s="6" t="s">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="J16" s="5"/>
       <c r="K16" s="5"/>
@@ -3488,31 +3185,31 @@
     </row>
     <row r="17" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
-        <v>118</v>
+        <v>100</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>106</v>
+        <v>88</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>107</v>
+        <v>89</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>119</v>
+        <v>101</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>120</v>
+        <v>102</v>
       </c>
       <c r="J17" s="5"/>
       <c r="K17" s="5"/>
@@ -3529,25 +3226,25 @@
     </row>
     <row r="18" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
-        <v>121</v>
+        <v>103</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>122</v>
+        <v>104</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>123</v>
+        <v>105</v>
       </c>
       <c r="H18" s="7"/>
       <c r="I18" s="7"/>
@@ -3566,31 +3263,31 @@
     </row>
     <row r="19" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
-        <v>124</v>
+        <v>106</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>122</v>
+        <v>104</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>123</v>
+        <v>105</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>125</v>
+        <v>107</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>126</v>
+        <v>108</v>
       </c>
       <c r="J19" s="5"/>
       <c r="K19" s="5"/>
@@ -3607,31 +3304,31 @@
     </row>
     <row r="20" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
-        <v>127</v>
+        <v>109</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>122</v>
+        <v>104</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>123</v>
+        <v>105</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>128</v>
+        <v>110</v>
       </c>
       <c r="I20" s="6" t="s">
-        <v>129</v>
+        <v>111</v>
       </c>
       <c r="J20" s="5"/>
       <c r="K20" s="5"/>
@@ -3648,31 +3345,31 @@
     </row>
     <row r="21" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
-        <v>130</v>
+        <v>112</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>122</v>
+        <v>104</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>123</v>
+        <v>105</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>131</v>
+        <v>113</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>132</v>
+        <v>114</v>
       </c>
       <c r="J21" s="5"/>
       <c r="K21" s="5"/>
@@ -3689,25 +3386,25 @@
     </row>
     <row r="22" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
-        <v>133</v>
+        <v>115</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>134</v>
+        <v>116</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>135</v>
+        <v>117</v>
       </c>
       <c r="H22" s="7"/>
       <c r="I22" s="7"/>
@@ -3726,31 +3423,31 @@
     </row>
     <row r="23" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>134</v>
+        <v>116</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>135</v>
+        <v>117</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>137</v>
+        <v>119</v>
       </c>
       <c r="I23" s="6" t="s">
-        <v>138</v>
+        <v>120</v>
       </c>
       <c r="J23" s="5"/>
       <c r="K23" s="5"/>
@@ -3767,31 +3464,31 @@
     </row>
     <row r="24" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
-        <v>139</v>
+        <v>121</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>134</v>
+        <v>116</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>135</v>
+        <v>117</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>140</v>
+        <v>122</v>
       </c>
       <c r="I24" s="6" t="s">
-        <v>141</v>
+        <v>123</v>
       </c>
       <c r="J24" s="5"/>
       <c r="K24" s="5"/>
@@ -3808,31 +3505,31 @@
     </row>
     <row r="25" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
-        <v>142</v>
+        <v>124</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>134</v>
+        <v>116</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>135</v>
+        <v>117</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>143</v>
+        <v>125</v>
       </c>
       <c r="I25" s="6" t="s">
-        <v>144</v>
+        <v>126</v>
       </c>
       <c r="J25" s="6"/>
       <c r="K25" s="5"/>
@@ -3849,25 +3546,25 @@
     </row>
     <row r="26" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
-        <v>145</v>
+        <v>127</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>146</v>
+        <v>128</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>147</v>
+        <v>129</v>
       </c>
       <c r="H26" s="5"/>
       <c r="I26" s="5"/>
@@ -3886,31 +3583,31 @@
     </row>
     <row r="27" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
-        <v>148</v>
+        <v>130</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>146</v>
+        <v>128</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>147</v>
+        <v>129</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>149</v>
+        <v>131</v>
       </c>
       <c r="I27" s="6" t="s">
-        <v>150</v>
+        <v>132</v>
       </c>
       <c r="J27" s="5"/>
       <c r="K27" s="5"/>
@@ -3927,31 +3624,31 @@
     </row>
     <row r="28" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
-        <v>151</v>
+        <v>133</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>146</v>
+        <v>128</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>147</v>
+        <v>129</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>152</v>
+        <v>134</v>
       </c>
       <c r="I28" s="6" t="s">
-        <v>152</v>
+        <v>134</v>
       </c>
       <c r="J28" s="5"/>
       <c r="K28" s="5"/>
@@ -3968,25 +3665,25 @@
     </row>
     <row r="29" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
-        <v>153</v>
+        <v>135</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>154</v>
+        <v>136</v>
       </c>
       <c r="G29" s="6" t="s">
-        <v>154</v>
+        <v>136</v>
       </c>
       <c r="H29" s="7"/>
       <c r="I29" s="7"/>
@@ -4005,31 +3702,31 @@
     </row>
     <row r="30" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
-        <v>155</v>
+        <v>137</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>154</v>
+        <v>136</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>154</v>
+        <v>136</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>156</v>
+        <v>138</v>
       </c>
       <c r="I30" s="6" t="s">
-        <v>157</v>
+        <v>139</v>
       </c>
       <c r="J30" s="5"/>
       <c r="K30" s="5"/>
@@ -4046,31 +3743,31 @@
     </row>
     <row r="31" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
-        <v>158</v>
+        <v>140</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>154</v>
+        <v>136</v>
       </c>
       <c r="G31" s="6" t="s">
-        <v>154</v>
+        <v>136</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>159</v>
+        <v>141</v>
       </c>
       <c r="I31" s="6" t="s">
-        <v>159</v>
+        <v>141</v>
       </c>
       <c r="J31" s="5"/>
       <c r="K31" s="5"/>
@@ -4087,25 +3784,25 @@
     </row>
     <row r="32" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
-        <v>160</v>
+        <v>142</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>161</v>
+        <v>143</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>162</v>
+        <v>144</v>
       </c>
       <c r="H32" s="7"/>
       <c r="I32" s="7"/>
@@ -4124,31 +3821,31 @@
     </row>
     <row r="33" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
-        <v>163</v>
+        <v>145</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>161</v>
+        <v>143</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>162</v>
+        <v>144</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>164</v>
+        <v>146</v>
       </c>
       <c r="I33" s="6" t="s">
-        <v>165</v>
+        <v>147</v>
       </c>
       <c r="J33" s="5"/>
       <c r="K33" s="5"/>
@@ -4165,31 +3862,31 @@
     </row>
     <row r="34" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
-        <v>166</v>
+        <v>148</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>161</v>
+        <v>143</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>162</v>
+        <v>144</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>167</v>
+        <v>149</v>
       </c>
       <c r="I34" s="6" t="s">
-        <v>168</v>
+        <v>150</v>
       </c>
       <c r="J34" s="5"/>
       <c r="K34" s="5"/>
@@ -4206,25 +3903,25 @@
     </row>
     <row r="35" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
-        <v>169</v>
+        <v>151</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>170</v>
+        <v>152</v>
       </c>
       <c r="G35" s="6" t="s">
-        <v>170</v>
+        <v>152</v>
       </c>
       <c r="H35" s="5"/>
       <c r="I35" s="5"/>
@@ -4243,31 +3940,31 @@
     </row>
     <row r="36" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
-        <v>171</v>
+        <v>153</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>170</v>
+        <v>152</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>170</v>
+        <v>152</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>172</v>
+        <v>154</v>
       </c>
       <c r="I36" s="6" t="s">
-        <v>173</v>
+        <v>155</v>
       </c>
       <c r="J36" s="5"/>
       <c r="K36" s="5"/>
@@ -4284,31 +3981,31 @@
     </row>
     <row r="37" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
-        <v>174</v>
+        <v>156</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F37" s="6" t="s">
-        <v>170</v>
+        <v>152</v>
       </c>
       <c r="G37" s="6" t="s">
-        <v>170</v>
+        <v>152</v>
       </c>
       <c r="H37" s="6" t="s">
-        <v>175</v>
+        <v>157</v>
       </c>
       <c r="I37" s="6" t="s">
-        <v>176</v>
+        <v>158</v>
       </c>
       <c r="J37" s="5"/>
       <c r="K37" s="5"/>
@@ -4325,25 +4022,25 @@
     </row>
     <row r="38" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="4" t="s">
-        <v>177</v>
+        <v>159</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F38" s="6" t="s">
-        <v>178</v>
+        <v>160</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>178</v>
+        <v>160</v>
       </c>
       <c r="H38" s="7"/>
       <c r="I38" s="7"/>
@@ -4362,31 +4059,31 @@
     </row>
     <row r="39" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="4" t="s">
-        <v>179</v>
+        <v>161</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F39" s="6" t="s">
-        <v>178</v>
+        <v>160</v>
       </c>
       <c r="G39" s="6" t="s">
-        <v>178</v>
+        <v>160</v>
       </c>
       <c r="H39" s="6" t="s">
-        <v>180</v>
+        <v>162</v>
       </c>
       <c r="I39" s="6" t="s">
-        <v>181</v>
+        <v>163</v>
       </c>
       <c r="J39" s="5"/>
       <c r="K39" s="5"/>
@@ -4403,25 +4100,25 @@
     </row>
     <row r="40" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
-        <v>182</v>
+        <v>164</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F40" s="6" t="s">
-        <v>183</v>
+        <v>165</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>184</v>
+        <v>166</v>
       </c>
       <c r="H40" s="7"/>
       <c r="I40" s="7"/>
@@ -4440,31 +4137,31 @@
     </row>
     <row r="41" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="4" t="s">
-        <v>185</v>
+        <v>167</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="F41" s="6" t="s">
-        <v>183</v>
+        <v>165</v>
       </c>
       <c r="G41" s="6" t="s">
-        <v>184</v>
+        <v>166</v>
       </c>
       <c r="H41" s="6" t="s">
-        <v>186</v>
+        <v>168</v>
       </c>
       <c r="I41" s="6" t="s">
-        <v>187</v>
+        <v>169</v>
       </c>
       <c r="J41" s="5"/>
       <c r="K41" s="5"/>
@@ -4481,19 +4178,19 @@
     </row>
     <row r="42" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="4" t="s">
-        <v>188</v>
+        <v>170</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>189</v>
+        <v>171</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>190</v>
+        <v>172</v>
       </c>
       <c r="F42" s="5"/>
       <c r="G42" s="5"/>
@@ -4501,11 +4198,11 @@
       <c r="I42" s="7"/>
       <c r="J42" s="5"/>
       <c r="K42" s="5"/>
-      <c r="L42" s="13" t="s">
-        <v>237</v>
-      </c>
-      <c r="M42" s="13" t="s">
-        <v>240</v>
+      <c r="L42" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="M42" s="12" t="s">
+        <v>217</v>
       </c>
       <c r="N42" s="5"/>
       <c r="O42" s="5"/>
@@ -4518,25 +4215,25 @@
     </row>
     <row r="43" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="4" t="s">
-        <v>191</v>
+        <v>173</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>189</v>
+        <v>171</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>190</v>
+        <v>172</v>
       </c>
       <c r="F43" s="6" t="s">
-        <v>192</v>
+        <v>174</v>
       </c>
       <c r="G43" s="6" t="s">
-        <v>193</v>
+        <v>175</v>
       </c>
       <c r="H43" s="5"/>
       <c r="I43" s="5"/>
@@ -4555,25 +4252,25 @@
     </row>
     <row r="44" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
-        <v>194</v>
+        <v>176</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>189</v>
+        <v>171</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>190</v>
+        <v>172</v>
       </c>
       <c r="F44" s="6" t="s">
-        <v>146</v>
+        <v>128</v>
       </c>
       <c r="G44" s="6" t="s">
-        <v>147</v>
+        <v>129</v>
       </c>
       <c r="H44" s="7"/>
       <c r="I44" s="7"/>
@@ -4592,25 +4289,25 @@
     </row>
     <row r="45" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="4" t="s">
-        <v>195</v>
+        <v>177</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>189</v>
+        <v>171</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>190</v>
+        <v>172</v>
       </c>
       <c r="F45" s="6" t="s">
-        <v>196</v>
+        <v>178</v>
       </c>
       <c r="G45" s="6" t="s">
-        <v>197</v>
+        <v>179</v>
       </c>
       <c r="H45" s="5"/>
       <c r="I45" s="5"/>
@@ -4629,25 +4326,25 @@
     </row>
     <row r="46" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="4" t="s">
-        <v>198</v>
+        <v>180</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>189</v>
+        <v>171</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>190</v>
+        <v>172</v>
       </c>
       <c r="F46" s="6" t="s">
-        <v>199</v>
+        <v>181</v>
       </c>
       <c r="G46" s="6" t="s">
-        <v>200</v>
+        <v>182</v>
       </c>
       <c r="H46" s="7"/>
       <c r="I46" s="7"/>
@@ -4666,19 +4363,19 @@
     </row>
     <row r="47" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="4" t="s">
-        <v>201</v>
+        <v>183</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>202</v>
+        <v>184</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>203</v>
+        <v>185</v>
       </c>
       <c r="F47" s="5"/>
       <c r="G47" s="5"/>
@@ -4686,11 +4383,11 @@
       <c r="I47" s="7"/>
       <c r="J47" s="5"/>
       <c r="K47" s="5"/>
-      <c r="L47" s="13" t="s">
-        <v>238</v>
-      </c>
-      <c r="M47" s="13" t="s">
-        <v>239</v>
+      <c r="L47" s="12" t="s">
+        <v>215</v>
+      </c>
+      <c r="M47" s="12" t="s">
+        <v>216</v>
       </c>
       <c r="N47" s="5"/>
       <c r="O47" s="5"/>
@@ -4703,25 +4400,25 @@
     </row>
     <row r="48" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="4" t="s">
-        <v>204</v>
+        <v>186</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>202</v>
+        <v>184</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>203</v>
+        <v>185</v>
       </c>
       <c r="F48" s="6" t="s">
-        <v>205</v>
+        <v>187</v>
       </c>
       <c r="G48" s="6" t="s">
-        <v>206</v>
+        <v>188</v>
       </c>
       <c r="H48" s="7"/>
       <c r="I48" s="7"/>
@@ -4740,25 +4437,25 @@
     </row>
     <row r="49" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="4" t="s">
-        <v>207</v>
+        <v>189</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>202</v>
+        <v>184</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>203</v>
+        <v>185</v>
       </c>
       <c r="F49" s="6" t="s">
-        <v>208</v>
+        <v>190</v>
       </c>
       <c r="G49" s="6" t="s">
-        <v>209</v>
+        <v>191</v>
       </c>
       <c r="H49" s="7"/>
       <c r="I49" s="7"/>
@@ -4777,25 +4474,25 @@
     </row>
     <row r="50" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
-        <v>210</v>
+        <v>192</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>202</v>
+        <v>184</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>203</v>
+        <v>185</v>
       </c>
       <c r="F50" s="6" t="s">
-        <v>211</v>
+        <v>193</v>
       </c>
       <c r="G50" s="6" t="s">
-        <v>212</v>
+        <v>194</v>
       </c>
       <c r="H50" s="7"/>
       <c r="I50" s="7"/>
@@ -4814,25 +4511,25 @@
     </row>
     <row r="51" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="4" t="s">
-        <v>213</v>
+        <v>195</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>202</v>
+        <v>184</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>203</v>
+        <v>185</v>
       </c>
       <c r="F51" s="6" t="s">
-        <v>214</v>
+        <v>196</v>
       </c>
       <c r="G51" s="6" t="s">
-        <v>214</v>
+        <v>196</v>
       </c>
       <c r="H51" s="7"/>
       <c r="I51" s="7"/>
@@ -4851,19 +4548,19 @@
     </row>
     <row r="52" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="4" t="s">
-        <v>215</v>
+        <v>197</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>216</v>
+        <v>198</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>217</v>
+        <v>199</v>
       </c>
       <c r="F52" s="5"/>
       <c r="G52" s="5"/>
@@ -4884,25 +4581,25 @@
     </row>
     <row r="53" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="4" t="s">
-        <v>218</v>
+        <v>200</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>216</v>
+        <v>198</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>217</v>
+        <v>199</v>
       </c>
       <c r="F53" s="6" t="s">
-        <v>219</v>
+        <v>201</v>
       </c>
       <c r="G53" s="6" t="s">
-        <v>220</v>
+        <v>202</v>
       </c>
       <c r="H53" s="5"/>
       <c r="I53" s="5"/>
@@ -4921,25 +4618,25 @@
     </row>
     <row r="54" spans="1:21" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="4" t="s">
-        <v>221</v>
+        <v>203</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>216</v>
+        <v>198</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>217</v>
+        <v>199</v>
       </c>
       <c r="F54" s="6" t="s">
-        <v>222</v>
+        <v>204</v>
       </c>
       <c r="G54" s="6" t="s">
-        <v>223</v>
+        <v>205</v>
       </c>
       <c r="H54" s="7"/>
       <c r="I54" s="7"/>

</xml_diff>